<commit_message>
Add EIC AUT notebooks and no-LQCD outputs
</commit_message>
<xml_diff>
--- a/Main/AUT_EEC_results/AUT_EEC_SIDIS_a0.01_b0.01_x0.01_Q100_LO.xlsx
+++ b/Main/AUT_EEC_results/AUT_EEC_SIDIS_a0.01_b0.01_x0.01_Q100_LO.xlsx
@@ -455,10 +455,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0005450203285390328</v>
+        <v>0.0002516442422594859</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0005450203285390328</v>
+        <v>0.0002516442422594859</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -469,10 +469,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0.001483463597042016</v>
+        <v>0.0007028951515155084</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001483463597042016</v>
+        <v>0.0007028951515155084</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -483,10 +483,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0.003055139777980665</v>
+        <v>0.00144247809354358</v>
       </c>
       <c r="C4" t="n">
-        <v>0.003055139777980665</v>
+        <v>0.00144247809354358</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -497,10 +497,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>0.004054684581511111</v>
+        <v>0.001917270044989975</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004054684581511111</v>
+        <v>0.001917270044989975</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -511,10 +511,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.003853327998439831</v>
+        <v>0.00181846597155239</v>
       </c>
       <c r="C6" t="n">
-        <v>0.003853327998439831</v>
+        <v>0.00181846597155239</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -525,10 +525,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>0.003409361332377388</v>
+        <v>0.001611032210414728</v>
       </c>
       <c r="C7" t="n">
-        <v>0.003409361332377388</v>
+        <v>0.001611032210414728</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -539,10 +539,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.003021085608700722</v>
+        <v>0.001430523248144156</v>
       </c>
       <c r="C8" t="n">
-        <v>0.003021085608700722</v>
+        <v>0.001430523248144156</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -553,10 +553,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>0.002765559107952385</v>
+        <v>0.001310202389223061</v>
       </c>
       <c r="C9" t="n">
-        <v>0.002765559107952385</v>
+        <v>0.001310202389223061</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>

</xml_diff>